<commit_message>
Update attendance system to properly enable fourth period attendance
Modify attendance and simple form templates to correctly handle fourth period attendance by disabling lunch period functionality and enabling fourth period as a regular class session.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7e4046e9-32b7-4838-9b98-49020ffa1c80
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: fe303809-30af-48e1-8706-02a5716f30c2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/3a213c01-649d-4274-bf74-8c5b6c6afe98/7e4046e9-32b7-4838-9b98-49020ffa1c80/2jWt9gH
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C552"/>
+  <dimension ref="A1:C554"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>336</t>
         </is>
       </c>
     </row>
@@ -463,7 +463,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>317</t>
+          <t>311</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>325</t>
+          <t>329</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>407</t>
+          <t>301</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>290</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>337</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>351</t>
+          <t>321</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>189</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>147</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>159</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>354</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>288</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>280</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>288</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>284</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>316</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>165</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>118</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>188</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>217</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>153</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>197</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>157</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>123</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>139</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>377</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>160</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>139</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>193</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>392</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>276</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>291</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>240</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>315</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>327</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>302</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>344</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>406</t>
+          <t>383</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>125</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>290</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>328</t>
+          <t>276</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>146</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>386</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>155</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>297</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>118</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>349</t>
+          <t>304</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>115</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>293</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>162</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>152</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>327</t>
+          <t>409</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>337</t>
+          <t>300</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>214</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>231</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>169</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>328</t>
+          <t>410</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>144</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>407</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>141</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>334</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>336</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>134</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>176</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>370</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>163</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>298</t>
+          <t>331</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>220</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>151</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>320</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>139</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>406</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>182</t>
+          <t>127</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>325</t>
+          <t>359</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>167</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>172</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>172</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>113</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>306</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>279</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>195</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>192</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>281</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>170</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>333</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>159</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>360</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>272</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>186</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>191</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>402</t>
+          <t>380</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>307</t>
+          <t>298</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>405</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>299</t>
+          <t>358</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>168</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>281</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>325</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>186</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>122</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>295</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>327</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>382</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>119</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>294</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>385</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>230</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>309</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>277</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>145</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2503,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>297</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>241</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>149</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2554,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>348</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>394</t>
+          <t>280</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>390</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>221</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2622,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>344</t>
+          <t>394</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>156</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>149</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>371</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>193</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>198</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>322</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>144</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>317</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>235</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>369</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>187</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>301</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>240</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>389</t>
+          <t>283</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>197</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>209</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>376</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>182</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>394</t>
+          <t>362</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>121</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>289</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>154</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>237</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>234</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>289</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>170</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3098,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>355</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>201</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>363</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>273</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>182</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>199</t>
         </is>
       </c>
     </row>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>312</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>203</t>
         </is>
       </c>
     </row>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>392</t>
+          <t>360</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>397</t>
+          <t>299</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>237</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>196</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>150</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>218</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>341</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>219</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>343</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>299</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>178</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>214</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3455,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>174</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>206</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>118</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>128</t>
         </is>
       </c>
     </row>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>346</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3540,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>135</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>347</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>293</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>214</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>396</t>
+          <t>368</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>382</t>
+          <t>357</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>218</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>194</t>
         </is>
       </c>
     </row>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>157</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>358</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>125</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>223</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>138</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3778,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>364</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3795,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>368</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>239</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>330</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>220</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>121</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>318</t>
+          <t>373</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>278</t>
         </is>
       </c>
     </row>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>377</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>395</t>
+          <t>287</t>
         </is>
       </c>
     </row>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>222</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>166</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>133</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>215</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>173</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>164</t>
         </is>
       </c>
     </row>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>116</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>226</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>198</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>328</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>305</t>
+          <t>323</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>131</t>
         </is>
       </c>
     </row>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>196</t>
         </is>
       </c>
     </row>
@@ -4169,7 +4169,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>133</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>365</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>171</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>195</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>122</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4254,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>285</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>124</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>121</t>
         </is>
       </c>
     </row>
@@ -4305,7 +4305,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>344</t>
+          <t>300</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4322,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>174</t>
         </is>
       </c>
     </row>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>223</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>213</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>187</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>177</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>307</t>
+          <t>388</t>
         </is>
       </c>
     </row>
@@ -4424,7 +4424,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>135</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>367</t>
         </is>
       </c>
     </row>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>352</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4492,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>202</t>
         </is>
       </c>
     </row>
@@ -4509,7 +4509,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>326</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>308</t>
+          <t>389</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>166</t>
+          <t>219</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>230</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>362</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>370</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>177</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>215</t>
         </is>
       </c>
     </row>
@@ -4662,7 +4662,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>239</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>351</t>
+          <t>316</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4696,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>151</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>225</t>
         </is>
       </c>
     </row>
@@ -4747,7 +4747,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>222</t>
         </is>
       </c>
     </row>
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>345</t>
+          <t>395</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>154</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>309</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>166</t>
         </is>
       </c>
     </row>
@@ -4849,7 +4849,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>148</t>
         </is>
       </c>
     </row>
@@ -4866,7 +4866,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>348</t>
+          <t>397</t>
         </is>
       </c>
     </row>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>154</t>
         </is>
       </c>
     </row>
@@ -4900,7 +4900,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>378</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>166</t>
+          <t>207</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>312</t>
         </is>
       </c>
     </row>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>196</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>186</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>346</t>
+          <t>313</t>
         </is>
       </c>
     </row>
@@ -5019,7 +5019,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>170</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>185</t>
+          <t>175</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>298</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>232</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>339</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>223</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>407</t>
+          <t>303</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>284</t>
         </is>
       </c>
     </row>
@@ -5155,7 +5155,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>241</t>
         </is>
       </c>
     </row>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>319</t>
+          <t>272</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>211</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>232</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5223,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>339</t>
+          <t>321</t>
         </is>
       </c>
     </row>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>182</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>212</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>155</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>382</t>
+          <t>279</t>
         </is>
       </c>
     </row>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>326</t>
         </is>
       </c>
     </row>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>349</t>
+          <t>299</t>
         </is>
       </c>
     </row>
@@ -5342,7 +5342,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>299</t>
+          <t>273</t>
         </is>
       </c>
     </row>
@@ -5359,7 +5359,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>160</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>296</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>384</t>
         </is>
       </c>
     </row>
@@ -5410,7 +5410,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>158</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>183</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>387</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>311</t>
         </is>
       </c>
     </row>
@@ -5478,7 +5478,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>193</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>136</t>
         </is>
       </c>
     </row>
@@ -5512,7 +5512,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>181</t>
         </is>
       </c>
     </row>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>140</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>396</t>
         </is>
       </c>
     </row>
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>169</t>
         </is>
       </c>
     </row>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>137</t>
         </is>
       </c>
     </row>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>318</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>329</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>130</t>
         </is>
       </c>
     </row>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>319</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5716,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>352</t>
         </is>
       </c>
     </row>
@@ -5733,7 +5733,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>345</t>
+          <t>301</t>
         </is>
       </c>
     </row>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>356</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5767,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>337</t>
+          <t>334</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>138</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>296</t>
         </is>
       </c>
     </row>
@@ -5818,7 +5818,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>345</t>
+          <t>310</t>
         </is>
       </c>
     </row>
@@ -5835,7 +5835,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>197</t>
         </is>
       </c>
     </row>
@@ -5852,7 +5852,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>299</t>
         </is>
       </c>
     </row>
@@ -5869,7 +5869,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>312</t>
         </is>
       </c>
     </row>
@@ -5886,7 +5886,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>119</t>
         </is>
       </c>
     </row>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>182</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5920,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204</t>
         </is>
       </c>
     </row>
@@ -5937,7 +5937,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>114</t>
         </is>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>193</t>
         </is>
       </c>
     </row>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>345</t>
         </is>
       </c>
     </row>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>120</t>
         </is>
       </c>
     </row>
@@ -6005,7 +6005,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>123</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>216</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>175</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>225</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>375</t>
+          <t>349</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>277</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>190</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>318</t>
+          <t>310</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>168</t>
         </is>
       </c>
     </row>
@@ -6158,7 +6158,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>210</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>120</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6192,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>217</t>
         </is>
       </c>
     </row>
@@ -6209,7 +6209,7 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>319</t>
         </is>
       </c>
     </row>
@@ -6226,7 +6226,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>130</t>
         </is>
       </c>
     </row>
@@ -6243,7 +6243,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>393</t>
+          <t>361</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6277,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>188</t>
         </is>
       </c>
     </row>
@@ -6294,7 +6294,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>189</t>
         </is>
       </c>
     </row>
@@ -6311,7 +6311,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>314</t>
         </is>
       </c>
     </row>
@@ -6328,7 +6328,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>224</t>
         </is>
       </c>
     </row>
@@ -6345,7 +6345,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>129</t>
         </is>
       </c>
     </row>
@@ -6362,7 +6362,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>234</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>235</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6413,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>361</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>228</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>164</t>
         </is>
       </c>
     </row>
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>236</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>184</t>
         </is>
       </c>
     </row>
@@ -6532,7 +6532,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>348</t>
+          <t>317</t>
         </is>
       </c>
     </row>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>335</t>
+          <t>332</t>
         </is>
       </c>
     </row>
@@ -6566,7 +6566,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>131</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>238</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>238</t>
         </is>
       </c>
     </row>
@@ -6617,7 +6617,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>319</t>
+          <t>374</t>
         </is>
       </c>
     </row>
@@ -6634,7 +6634,7 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>409</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>158</t>
         </is>
       </c>
     </row>
@@ -6668,7 +6668,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>295</t>
         </is>
       </c>
     </row>
@@ -6685,7 +6685,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>376</t>
         </is>
       </c>
     </row>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>375</t>
+          <t>307</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>395</t>
+          <t>363</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>177</t>
+          <t>113</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>321</t>
         </is>
       </c>
     </row>
@@ -6770,7 +6770,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>392</t>
+          <t>372</t>
         </is>
       </c>
     </row>
@@ -6787,7 +6787,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>129</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6804,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>187</t>
         </is>
       </c>
     </row>
@@ -6821,7 +6821,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>366</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>174</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>182</t>
+          <t>191</t>
         </is>
       </c>
     </row>
@@ -6872,7 +6872,7 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>231</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>335</t>
+          <t>293</t>
         </is>
       </c>
     </row>
@@ -6906,7 +6906,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>165</t>
         </is>
       </c>
     </row>
@@ -6918,12 +6918,12 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>이준익</t>
+          <t>김예승</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>351</t>
         </is>
       </c>
     </row>
@@ -6940,7 +6940,7 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>158</t>
         </is>
       </c>
     </row>
@@ -6957,7 +6957,7 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>276</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6974,7 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>402</t>
+          <t>324</t>
         </is>
       </c>
     </row>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>142</t>
         </is>
       </c>
     </row>
@@ -7025,7 +7025,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>375</t>
         </is>
       </c>
     </row>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>393</t>
+          <t>371</t>
         </is>
       </c>
     </row>
@@ -7059,7 +7059,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>348</t>
+          <t>323</t>
         </is>
       </c>
     </row>
@@ -7076,7 +7076,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>141</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7093,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>397</t>
+          <t>333</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7110,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>307</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>185</t>
         </is>
       </c>
     </row>
@@ -7144,7 +7144,7 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>338</t>
         </is>
       </c>
     </row>
@@ -7161,7 +7161,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>126</t>
         </is>
       </c>
     </row>
@@ -7195,7 +7195,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>374</t>
+          <t>379</t>
         </is>
       </c>
     </row>
@@ -7212,7 +7212,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>224</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>331</t>
+          <t>290</t>
         </is>
       </c>
     </row>
@@ -7246,7 +7246,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>205</t>
         </is>
       </c>
     </row>
@@ -7280,7 +7280,7 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>168</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7297,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>285</t>
         </is>
       </c>
     </row>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>118</t>
         </is>
       </c>
     </row>
@@ -7326,12 +7326,12 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>진승현</t>
+          <t>최서윤</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>115</t>
         </is>
       </c>
     </row>
@@ -7348,7 +7348,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>342</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>208</t>
         </is>
       </c>
     </row>
@@ -7382,7 +7382,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>305</t>
         </is>
       </c>
     </row>
@@ -7399,7 +7399,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>233</t>
         </is>
       </c>
     </row>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>291</t>
         </is>
       </c>
     </row>
@@ -7433,7 +7433,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>376</t>
+          <t>353</t>
         </is>
       </c>
     </row>
@@ -7450,7 +7450,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>378</t>
+          <t>354</t>
         </is>
       </c>
     </row>
@@ -7467,7 +7467,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>272</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>117</t>
         </is>
       </c>
     </row>
@@ -7501,7 +7501,7 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>297</t>
         </is>
       </c>
     </row>
@@ -7518,7 +7518,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>161</t>
         </is>
       </c>
     </row>
@@ -7552,7 +7552,7 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>356</t>
         </is>
       </c>
     </row>
@@ -7569,7 +7569,7 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>229</t>
         </is>
       </c>
     </row>
@@ -7603,7 +7603,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>320</t>
         </is>
       </c>
     </row>
@@ -7620,7 +7620,7 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>177</t>
+          <t>221</t>
         </is>
       </c>
     </row>
@@ -7637,7 +7637,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>143</t>
         </is>
       </c>
     </row>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>227</t>
         </is>
       </c>
     </row>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>173</t>
         </is>
       </c>
     </row>
@@ -7705,7 +7705,7 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>353</t>
         </is>
       </c>
     </row>
@@ -7722,7 +7722,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>132</t>
         </is>
       </c>
     </row>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>396</t>
+          <t>364</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>375</t>
         </is>
       </c>
     </row>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>135</t>
         </is>
       </c>
     </row>
@@ -7790,7 +7790,7 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>162</t>
         </is>
       </c>
     </row>
@@ -7807,7 +7807,7 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>344</t>
+          <t>338</t>
         </is>
       </c>
     </row>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>355</t>
         </is>
       </c>
     </row>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>153</t>
         </is>
       </c>
     </row>
@@ -7875,7 +7875,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>184</t>
         </is>
       </c>
     </row>
@@ -7892,7 +7892,7 @@
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>192</t>
         </is>
       </c>
     </row>
@@ -7909,7 +7909,7 @@
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>331</t>
+          <t>286</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>185</t>
         </is>
       </c>
     </row>
@@ -7943,7 +7943,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>127</t>
         </is>
       </c>
     </row>
@@ -7960,7 +7960,7 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>143</t>
         </is>
       </c>
     </row>
@@ -7977,7 +7977,7 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>178</t>
         </is>
       </c>
     </row>
@@ -7994,7 +7994,7 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>159</t>
         </is>
       </c>
     </row>
@@ -8011,7 +8011,7 @@
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>374</t>
         </is>
       </c>
     </row>
@@ -8028,7 +8028,7 @@
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>326</t>
+          <t>292</t>
         </is>
       </c>
     </row>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>305</t>
+          <t>287</t>
         </is>
       </c>
     </row>
@@ -8062,7 +8062,7 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>327</t>
+          <t>298</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>116</t>
         </is>
       </c>
     </row>
@@ -8096,7 +8096,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>346</t>
+          <t>284</t>
         </is>
       </c>
     </row>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>331</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8147,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>328</t>
         </is>
       </c>
     </row>
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>117</t>
         </is>
       </c>
     </row>
@@ -8181,7 +8181,7 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>132</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>339</t>
+          <t>411</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>128</t>
         </is>
       </c>
     </row>
@@ -8232,7 +8232,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>387</t>
+          <t>286</t>
         </is>
       </c>
     </row>
@@ -8249,7 +8249,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>134</t>
         </is>
       </c>
     </row>
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>125</t>
         </is>
       </c>
     </row>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>185</t>
+          <t>152</t>
         </is>
       </c>
     </row>
@@ -8317,7 +8317,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>140</t>
         </is>
       </c>
     </row>
@@ -8334,7 +8334,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>335</t>
         </is>
       </c>
     </row>
@@ -8351,7 +8351,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>366</t>
         </is>
       </c>
     </row>
@@ -8368,7 +8368,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>393</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>406</t>
         </is>
       </c>
     </row>
@@ -8419,7 +8419,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>179</t>
         </is>
       </c>
     </row>
@@ -8436,7 +8436,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>149</t>
         </is>
       </c>
     </row>
@@ -8453,7 +8453,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>314</t>
         </is>
       </c>
     </row>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>282</t>
         </is>
       </c>
     </row>
@@ -8487,7 +8487,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>155</t>
         </is>
       </c>
     </row>
@@ -8504,7 +8504,7 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>128</t>
         </is>
       </c>
     </row>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>271</t>
         </is>
       </c>
     </row>
@@ -8538,7 +8538,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>124</t>
         </is>
       </c>
     </row>
@@ -8555,7 +8555,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>233</t>
         </is>
       </c>
     </row>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>149</t>
         </is>
       </c>
     </row>
@@ -8589,7 +8589,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>326</t>
+          <t>408</t>
         </is>
       </c>
     </row>
@@ -8606,7 +8606,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>389</t>
+          <t>313</t>
         </is>
       </c>
     </row>
@@ -8623,7 +8623,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>317</t>
+          <t>372</t>
         </is>
       </c>
     </row>
@@ -8640,7 +8640,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>303</t>
         </is>
       </c>
     </row>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>308</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>369</t>
         </is>
       </c>
     </row>
@@ -8691,7 +8691,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>138</t>
         </is>
       </c>
     </row>
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>283</t>
         </is>
       </c>
     </row>
@@ -8725,7 +8725,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>156</t>
         </is>
       </c>
     </row>
@@ -8759,7 +8759,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>305</t>
         </is>
       </c>
     </row>
@@ -8776,7 +8776,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>378</t>
+          <t>308</t>
         </is>
       </c>
     </row>
@@ -8793,7 +8793,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>330</t>
         </is>
       </c>
     </row>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>195</t>
         </is>
       </c>
     </row>
@@ -8844,7 +8844,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>278</t>
         </is>
       </c>
     </row>
@@ -8861,7 +8861,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>325</t>
         </is>
       </c>
     </row>
@@ -8878,7 +8878,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>376</t>
+          <t>274</t>
         </is>
       </c>
     </row>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>406</t>
+          <t>277</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8912,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>381</t>
         </is>
       </c>
     </row>
@@ -8929,7 +8929,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>298</t>
+          <t>410</t>
         </is>
       </c>
     </row>
@@ -8946,7 +8946,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>131</t>
         </is>
       </c>
     </row>
@@ -8963,7 +8963,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>189</t>
         </is>
       </c>
     </row>
@@ -8980,7 +8980,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>367</t>
         </is>
       </c>
     </row>
@@ -8997,7 +8997,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>137</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>373</t>
         </is>
       </c>
     </row>
@@ -9048,7 +9048,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>391</t>
         </is>
       </c>
     </row>
@@ -9065,7 +9065,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>310</t>
         </is>
       </c>
     </row>
@@ -9082,7 +9082,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>121</t>
         </is>
       </c>
     </row>
@@ -9099,7 +9099,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>335</t>
         </is>
       </c>
     </row>
@@ -9116,7 +9116,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>146</t>
         </is>
       </c>
     </row>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>236</t>
         </is>
       </c>
     </row>
@@ -9150,7 +9150,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>176</t>
         </is>
       </c>
     </row>
@@ -9167,7 +9167,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>147</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>163</t>
         </is>
       </c>
     </row>
@@ -9201,7 +9201,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>164</t>
         </is>
       </c>
     </row>
@@ -9218,7 +9218,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>145</t>
         </is>
       </c>
     </row>
@@ -9235,7 +9235,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>304</t>
         </is>
       </c>
     </row>
@@ -9269,7 +9269,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>400</t>
         </is>
       </c>
     </row>
@@ -9286,7 +9286,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>216</t>
         </is>
       </c>
     </row>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>366</t>
         </is>
       </c>
     </row>
@@ -9337,7 +9337,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>275</t>
         </is>
       </c>
     </row>
@@ -9354,7 +9354,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>332</t>
         </is>
       </c>
     </row>
@@ -9371,7 +9371,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>308</t>
+          <t>273</t>
         </is>
       </c>
     </row>
@@ -9388,7 +9388,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>180</t>
         </is>
       </c>
     </row>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>171</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>141</t>
         </is>
       </c>
     </row>
@@ -9439,7 +9439,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>179</t>
         </is>
       </c>
     </row>
@@ -9502,12 +9502,12 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>김원중</t>
+          <t>남강민</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>282</t>
+          <t>322</t>
         </is>
       </c>
     </row>
@@ -9524,7 +9524,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>179</t>
         </is>
       </c>
     </row>
@@ -9541,7 +9541,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>116</t>
         </is>
       </c>
     </row>
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>289</t>
         </is>
       </c>
     </row>
@@ -9575,7 +9575,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>357</t>
         </is>
       </c>
     </row>
@@ -9626,7 +9626,7 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>374</t>
+          <t>337</t>
         </is>
       </c>
     </row>
@@ -9643,7 +9643,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>405</t>
         </is>
       </c>
     </row>
@@ -9660,7 +9660,7 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>232</t>
         </is>
       </c>
     </row>
@@ -9677,7 +9677,7 @@
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>142</t>
         </is>
       </c>
     </row>
@@ -9694,7 +9694,7 @@
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>180</t>
         </is>
       </c>
     </row>
@@ -9711,7 +9711,7 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>163</t>
         </is>
       </c>
     </row>
@@ -9728,7 +9728,7 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>340</t>
         </is>
       </c>
     </row>
@@ -9745,7 +9745,7 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>349</t>
+          <t>398</t>
         </is>
       </c>
     </row>
@@ -9762,7 +9762,7 @@
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>387</t>
+          <t>350</t>
         </is>
       </c>
     </row>
@@ -9779,7 +9779,7 @@
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>359</t>
         </is>
       </c>
     </row>
@@ -9796,7 +9796,41 @@
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>379</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>10329</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>유제인</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>10303</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>김지온</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>229</t>
         </is>
       </c>
     </row>

</xml_diff>